<commit_message>
Edit inside of this files
</commit_message>
<xml_diff>
--- a/APLOS/POPResources/Templates/Lvr20171Bengali.xlsx
+++ b/APLOS/POPResources/Templates/Lvr20171Bengali.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\APLOS.New\APLOS\POPResources\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Aplos.New\APLOS\POPResources\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427ADA54-9FBD-4E16-A9C9-582F64CE9695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -175,16 +176,16 @@
     <t>লায়লা স্টাইলস লিঃ</t>
   </si>
   <si>
-    <t xml:space="preserve">বাহাদুরপুর, সিকদার বাড়ী, গাজীপুর, বাংলাদেশ </t>
-  </si>
-  <si>
     <t xml:space="preserve">ফরমঃ ৯ [বাংলাদেশ শ্রম আইন ২০০৬ , ধারা -১০,১১৫,১১৬ ও ১১৭ এবং বাংলাদেশ শ্রম বিধিমালা ২০০৫, বিধি-২৪ ও ১০৮(১) ] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">বাহাদুরপুর, সিকদার বাড়ী, গাজীপুর, বাংলাদেশ  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-5000445]###0;"/>
     <numFmt numFmtId="165" formatCode="[$-5000445]#,##0_);\(#,##0\)"/>
@@ -436,110 +437,109 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="6" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -819,81 +819,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="1.140625" style="4" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="36" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" style="36" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" style="36" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="36" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="36" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" style="36" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" style="36" customWidth="1"/>
-    <col min="9" max="9" width="13" style="36" customWidth="1"/>
-    <col min="10" max="10" width="12.85546875" style="36" customWidth="1"/>
-    <col min="11" max="11" width="12.28515625" style="36" customWidth="1"/>
-    <col min="12" max="12" width="16.28515625" style="36" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" style="36" customWidth="1"/>
-    <col min="14" max="15" width="15.42578125" style="36" customWidth="1"/>
-    <col min="16" max="16" width="19.28515625" style="36" customWidth="1"/>
-    <col min="17" max="17" width="16" style="36" customWidth="1"/>
-    <col min="18" max="18" width="14" style="36" customWidth="1"/>
-    <col min="19" max="19" width="14.28515625" style="36" customWidth="1"/>
-    <col min="20" max="20" width="15.28515625" style="36" customWidth="1"/>
-    <col min="21" max="21" width="14.28515625" style="36" customWidth="1"/>
-    <col min="22" max="22" width="19.5703125" style="36" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="36"/>
+    <col min="1" max="1" width="1.109375" style="4" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="16" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="16" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="16" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" style="16" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="13" style="16" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" style="16" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" style="16" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="16" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" style="16" customWidth="1"/>
+    <col min="14" max="15" width="15.44140625" style="16" customWidth="1"/>
+    <col min="16" max="16" width="19.33203125" style="16" customWidth="1"/>
+    <col min="17" max="17" width="16" style="16" customWidth="1"/>
+    <col min="18" max="18" width="14" style="16" customWidth="1"/>
+    <col min="19" max="19" width="14.33203125" style="16" customWidth="1"/>
+    <col min="20" max="20" width="15.33203125" style="16" customWidth="1"/>
+    <col min="21" max="21" width="14.33203125" style="16" customWidth="1"/>
+    <col min="22" max="22" width="19.5546875" style="16" customWidth="1"/>
+    <col min="23" max="16384" width="9.109375" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="4" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" s="4" customFormat="1" ht="37.5" customHeight="1">
+      <c r="B2" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="S2" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+    </row>
+    <row r="3" spans="1:22" s="4" customFormat="1" ht="19.5" customHeight="1">
+      <c r="B3" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-    </row>
-    <row r="2" spans="1:22" s="4" customFormat="1" ht="37.5" customHeight="1">
-      <c r="B2" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="S2" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-    </row>
-    <row r="3" spans="1:22" s="4" customFormat="1" ht="19.5" customHeight="1">
-      <c r="B3" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-    </row>
-    <row r="4" spans="1:22" s="4" customFormat="1" ht="26.25">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+    </row>
+    <row r="4" spans="1:22" s="4" customFormat="1" ht="24.6">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -904,27 +896,27 @@
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="16" t="s">
+      <c r="Q4" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="17"/>
-      <c r="S4" s="15" t="s">
+      <c r="R4" s="34"/>
+      <c r="S4" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="T4" s="15"/>
-      <c r="U4" s="15"/>
-      <c r="V4" s="15"/>
-    </row>
-    <row r="5" spans="1:22" s="4" customFormat="1" ht="26.25">
+      <c r="T4" s="32"/>
+      <c r="U4" s="32"/>
+      <c r="V4" s="32"/>
+    </row>
+    <row r="5" spans="1:22" s="4" customFormat="1" ht="24.6">
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -935,16 +927,16 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
-      <c r="Q5" s="16" t="s">
+      <c r="Q5" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="R5" s="17"/>
-      <c r="S5" s="15" t="s">
+      <c r="R5" s="34"/>
+      <c r="S5" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
-      <c r="V5" s="15"/>
+      <c r="T5" s="32"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="32"/>
     </row>
     <row r="6" spans="1:22" s="4" customFormat="1">
       <c r="B6" s="5"/>
@@ -973,61 +965,61 @@
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="10" t="s">
+      <c r="E7" s="27"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="J7" s="13"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="27" t="s">
+      <c r="J7" s="27"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="M7" s="10" t="s">
+      <c r="M7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="N7" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="O7" s="10" t="s">
+      <c r="O7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="10" t="s">
+      <c r="P7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="Q7" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="13"/>
-      <c r="S7" s="14"/>
-      <c r="T7" s="25" t="s">
+      <c r="R7" s="27"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="U7" s="10" t="s">
+      <c r="U7" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="V7" s="10" t="s">
+      <c r="V7" s="22" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:22" s="4" customFormat="1" ht="54.75" customHeight="1">
-      <c r="B8" s="24"/>
-      <c r="C8" s="11"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1037,8 +1029,8 @@
       <c r="F8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="24"/>
-      <c r="H8" s="11"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="29"/>
       <c r="I8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1048,11 +1040,11 @@
       <c r="K8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L8" s="28"/>
-      <c r="M8" s="24"/>
-      <c r="N8" s="24"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="24"/>
+      <c r="L8" s="31"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="29"/>
+      <c r="P8" s="23"/>
       <c r="Q8" s="6" t="s">
         <v>18</v>
       </c>
@@ -1062,529 +1054,537 @@
       <c r="S8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="T8" s="26"/>
-      <c r="U8" s="24"/>
-      <c r="V8" s="24"/>
-    </row>
-    <row r="9" spans="1:22" s="34" customFormat="1">
+      <c r="T8" s="25"/>
+      <c r="U8" s="23"/>
+      <c r="V8" s="23"/>
+    </row>
+    <row r="9" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="30" t="s">
+      <c r="F9" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="30" t="s">
+      <c r="I9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="J9" s="30" t="s">
+      <c r="J9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="30" t="s">
+      <c r="K9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="L9" s="31" t="s">
+      <c r="L9" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="M9" s="32" t="s">
+      <c r="M9" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="N9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="O9" s="29" t="s">
+      <c r="O9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="P9" s="29" t="s">
+      <c r="P9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="Q9" s="30" t="s">
+      <c r="Q9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="R9" s="30" t="s">
+      <c r="R9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="S9" s="30" t="s">
+      <c r="S9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="T9" s="30"/>
-      <c r="U9" s="29"/>
-      <c r="V9" s="29"/>
-    </row>
-    <row r="10" spans="1:22" s="34" customFormat="1">
+      <c r="T9" s="10"/>
+      <c r="U9" s="9"/>
+      <c r="V9" s="9"/>
+    </row>
+    <row r="10" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A10" s="7"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
-      <c r="K10" s="33"/>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="33"/>
-      <c r="O10" s="33"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="33"/>
-      <c r="R10" s="35"/>
-      <c r="S10" s="33"/>
-      <c r="T10" s="33"/>
-      <c r="U10" s="33"/>
-      <c r="V10" s="33"/>
-    </row>
-    <row r="11" spans="1:22" s="34" customFormat="1">
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+    </row>
+    <row r="11" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A11" s="7"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="33"/>
-      <c r="J11" s="35"/>
-      <c r="K11" s="33"/>
-      <c r="L11" s="33"/>
-      <c r="M11" s="33"/>
-      <c r="N11" s="33"/>
-      <c r="O11" s="33"/>
-      <c r="P11" s="33"/>
-      <c r="Q11" s="33"/>
-      <c r="R11" s="35"/>
-      <c r="S11" s="33"/>
-      <c r="T11" s="33"/>
-      <c r="U11" s="33"/>
-      <c r="V11" s="33"/>
-    </row>
-    <row r="12" spans="1:22" s="34" customFormat="1">
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="15"/>
+      <c r="S11" s="13"/>
+      <c r="T11" s="13"/>
+      <c r="U11" s="13"/>
+      <c r="V11" s="13"/>
+    </row>
+    <row r="12" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A12" s="7"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="33"/>
-      <c r="O12" s="33"/>
-      <c r="P12" s="33"/>
-      <c r="Q12" s="33"/>
-      <c r="R12" s="33"/>
-      <c r="S12" s="33"/>
-      <c r="T12" s="33"/>
-      <c r="U12" s="33"/>
-      <c r="V12" s="33"/>
-    </row>
-    <row r="13" spans="1:22" s="34" customFormat="1">
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="13"/>
+      <c r="T12" s="13"/>
+      <c r="U12" s="13"/>
+      <c r="V12" s="13"/>
+    </row>
+    <row r="13" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A13" s="7"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33" t="s">
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="E13" s="33"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33" t="s">
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-    </row>
-    <row r="14" spans="1:22" s="34" customFormat="1">
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="13"/>
+      <c r="S13" s="13"/>
+      <c r="T13" s="13"/>
+      <c r="U13" s="13"/>
+      <c r="V13" s="13"/>
+    </row>
+    <row r="14" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A14" s="7"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="33"/>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
-      <c r="N14" s="33"/>
-      <c r="O14" s="33"/>
-      <c r="P14" s="33"/>
-      <c r="Q14" s="33"/>
-      <c r="R14" s="33"/>
-      <c r="S14" s="33"/>
-      <c r="T14" s="33"/>
-      <c r="U14" s="33"/>
-      <c r="V14" s="33"/>
-    </row>
-    <row r="15" spans="1:22" s="34" customFormat="1">
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="13"/>
+      <c r="S14" s="13"/>
+      <c r="T14" s="13"/>
+      <c r="U14" s="13"/>
+      <c r="V14" s="13"/>
+    </row>
+    <row r="15" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A15" s="7"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
-      <c r="N15" s="33"/>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33"/>
-      <c r="Q15" s="33"/>
-      <c r="R15" s="33"/>
-      <c r="S15" s="33"/>
-      <c r="T15" s="33"/>
-      <c r="U15" s="33"/>
-      <c r="V15" s="33"/>
-    </row>
-    <row r="16" spans="1:22" s="34" customFormat="1">
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13"/>
+      <c r="S15" s="13"/>
+      <c r="T15" s="13"/>
+      <c r="U15" s="13"/>
+      <c r="V15" s="13"/>
+    </row>
+    <row r="16" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A16" s="7"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
-      <c r="N16" s="33"/>
-      <c r="O16" s="33"/>
-      <c r="P16" s="33"/>
-      <c r="Q16" s="33"/>
-      <c r="R16" s="33"/>
-      <c r="S16" s="33"/>
-      <c r="T16" s="33"/>
-      <c r="U16" s="33"/>
-      <c r="V16" s="33"/>
-    </row>
-    <row r="17" spans="1:22" s="34" customFormat="1">
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
+      <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="13"/>
+      <c r="S16" s="13"/>
+      <c r="T16" s="13"/>
+      <c r="U16" s="13"/>
+      <c r="V16" s="13"/>
+    </row>
+    <row r="17" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A17" s="7"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
-      <c r="N17" s="33"/>
-      <c r="O17" s="33"/>
-      <c r="P17" s="33"/>
-      <c r="Q17" s="33"/>
-      <c r="R17" s="33"/>
-      <c r="S17" s="33"/>
-      <c r="T17" s="33"/>
-      <c r="U17" s="33"/>
-      <c r="V17" s="33"/>
-    </row>
-    <row r="18" spans="1:22" s="34" customFormat="1">
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+      <c r="T17" s="13"/>
+      <c r="U17" s="13"/>
+      <c r="V17" s="13"/>
+    </row>
+    <row r="18" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A18" s="7"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
-      <c r="N18" s="33"/>
-      <c r="O18" s="33"/>
-      <c r="P18" s="33"/>
-      <c r="Q18" s="33"/>
-      <c r="R18" s="33"/>
-      <c r="S18" s="33"/>
-      <c r="T18" s="33"/>
-      <c r="U18" s="33"/>
-      <c r="V18" s="33"/>
-    </row>
-    <row r="19" spans="1:22" s="34" customFormat="1">
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
+      <c r="V18" s="13"/>
+    </row>
+    <row r="19" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A19" s="7"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
-      <c r="N19" s="33"/>
-      <c r="O19" s="33"/>
-      <c r="P19" s="33"/>
-      <c r="Q19" s="33"/>
-      <c r="R19" s="33"/>
-      <c r="S19" s="33"/>
-      <c r="T19" s="33"/>
-      <c r="U19" s="33"/>
-      <c r="V19" s="33"/>
-    </row>
-    <row r="20" spans="1:22" s="34" customFormat="1">
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="13"/>
+      <c r="U19" s="13"/>
+      <c r="V19" s="13"/>
+    </row>
+    <row r="20" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A20" s="7"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="33"/>
-      <c r="J20" s="33"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="33"/>
-      <c r="M20" s="33"/>
-      <c r="N20" s="33"/>
-      <c r="O20" s="33"/>
-      <c r="P20" s="33"/>
-      <c r="Q20" s="33"/>
-      <c r="R20" s="33"/>
-      <c r="S20" s="33"/>
-      <c r="T20" s="33"/>
-      <c r="U20" s="33"/>
-      <c r="V20" s="33"/>
-    </row>
-    <row r="21" spans="1:22" s="34" customFormat="1">
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="13"/>
+      <c r="S20" s="13"/>
+      <c r="T20" s="13"/>
+      <c r="U20" s="13"/>
+      <c r="V20" s="13"/>
+    </row>
+    <row r="21" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A21" s="7"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
-      <c r="N21" s="33"/>
-      <c r="O21" s="33"/>
-      <c r="P21" s="33"/>
-      <c r="Q21" s="33"/>
-      <c r="R21" s="33"/>
-      <c r="S21" s="33"/>
-      <c r="T21" s="33"/>
-      <c r="U21" s="33"/>
-      <c r="V21" s="33"/>
-    </row>
-    <row r="22" spans="1:22" s="34" customFormat="1">
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="13"/>
+      <c r="V21" s="13"/>
+    </row>
+    <row r="22" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A22" s="7"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="33"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="33"/>
-      <c r="P22" s="33"/>
-      <c r="Q22" s="33"/>
-      <c r="R22" s="33"/>
-      <c r="S22" s="33"/>
-      <c r="T22" s="33"/>
-      <c r="U22" s="33"/>
-      <c r="V22" s="33"/>
-    </row>
-    <row r="23" spans="1:22" s="34" customFormat="1">
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="13"/>
+      <c r="V22" s="13"/>
+    </row>
+    <row r="23" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A23" s="7"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="33"/>
-      <c r="J23" s="33"/>
-      <c r="K23" s="33"/>
-      <c r="L23" s="33"/>
-      <c r="M23" s="33"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
-      <c r="P23" s="33"/>
-      <c r="Q23" s="33"/>
-      <c r="R23" s="33"/>
-      <c r="S23" s="33"/>
-      <c r="T23" s="33"/>
-      <c r="U23" s="33"/>
-      <c r="V23" s="33"/>
-    </row>
-    <row r="24" spans="1:22" s="34" customFormat="1">
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="13"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="13"/>
+      <c r="V23" s="13"/>
+    </row>
+    <row r="24" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A24" s="7"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="33"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="33"/>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33"/>
-      <c r="Q24" s="33"/>
-      <c r="R24" s="33"/>
-      <c r="S24" s="33"/>
-      <c r="T24" s="33"/>
-      <c r="U24" s="33"/>
-      <c r="V24" s="33"/>
-    </row>
-    <row r="25" spans="1:22" s="34" customFormat="1">
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="13"/>
+      <c r="T24" s="13"/>
+      <c r="U24" s="13"/>
+      <c r="V24" s="13"/>
+    </row>
+    <row r="25" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A25" s="7"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="33"/>
-      <c r="H25" s="33"/>
-      <c r="I25" s="33"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
-      <c r="M25" s="33"/>
-      <c r="N25" s="33"/>
-      <c r="O25" s="33"/>
-      <c r="P25" s="33"/>
-      <c r="Q25" s="33"/>
-      <c r="R25" s="33"/>
-      <c r="S25" s="33"/>
-      <c r="T25" s="33"/>
-      <c r="U25" s="33"/>
-      <c r="V25" s="33"/>
-    </row>
-    <row r="26" spans="1:22" s="34" customFormat="1">
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
+      <c r="P25" s="13"/>
+      <c r="Q25" s="13"/>
+      <c r="R25" s="13"/>
+      <c r="S25" s="13"/>
+      <c r="T25" s="13"/>
+      <c r="U25" s="13"/>
+      <c r="V25" s="13"/>
+    </row>
+    <row r="26" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A26" s="7"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="33"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
-      <c r="S26" s="33"/>
-      <c r="T26" s="33"/>
-      <c r="U26" s="33"/>
-      <c r="V26" s="33"/>
-    </row>
-    <row r="27" spans="1:22" s="34" customFormat="1">
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
+      <c r="Q26" s="13"/>
+      <c r="R26" s="13"/>
+      <c r="S26" s="13"/>
+      <c r="T26" s="13"/>
+      <c r="U26" s="13"/>
+      <c r="V26" s="13"/>
+    </row>
+    <row r="27" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A27" s="7"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="33"/>
-      <c r="I27" s="33"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
-      <c r="M27" s="33"/>
-      <c r="N27" s="33"/>
-      <c r="O27" s="33"/>
-      <c r="P27" s="33"/>
-      <c r="Q27" s="33"/>
-      <c r="R27" s="33"/>
-      <c r="S27" s="33"/>
-      <c r="T27" s="33"/>
-      <c r="U27" s="33"/>
-      <c r="V27" s="33"/>
-    </row>
-    <row r="28" spans="1:22" s="34" customFormat="1">
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="13"/>
+      <c r="S27" s="13"/>
+      <c r="T27" s="13"/>
+      <c r="U27" s="13"/>
+      <c r="V27" s="13"/>
+    </row>
+    <row r="28" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A28" s="7"/>
     </row>
-    <row r="29" spans="1:22" s="34" customFormat="1">
+    <row r="29" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A29" s="7"/>
     </row>
-    <row r="30" spans="1:22" s="34" customFormat="1">
+    <row r="30" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A30" s="7"/>
     </row>
-    <row r="31" spans="1:22" s="34" customFormat="1">
+    <row r="31" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A31" s="7"/>
     </row>
-    <row r="32" spans="1:22" s="34" customFormat="1">
+    <row r="32" spans="1:22" s="14" customFormat="1" ht="15">
       <c r="A32" s="7"/>
     </row>
-    <row r="33" spans="1:1" s="34" customFormat="1">
+    <row r="33" spans="1:1" s="14" customFormat="1" ht="15">
       <c r="A33" s="7"/>
     </row>
-    <row r="34" spans="1:1" s="34" customFormat="1">
+    <row r="34" spans="1:1" s="14" customFormat="1" ht="15">
       <c r="A34" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="S4:V4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="S5:V5"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="S2:V2"/>
@@ -1601,14 +1601,6 @@
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="S4:V4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="Q5:R5"/>
-    <mergeCell ref="S5:V5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>